<commit_message>
Supplier and Category Analysis
</commit_message>
<xml_diff>
--- a/Excel/Procurement KPI Analysis Dataset.xlsx
+++ b/Excel/Procurement KPI Analysis Dataset.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gebre\Desktop\Purchase-Order-Performance-Analysis\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D72444-5B16-4ECA-B13D-BCD251FB461F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7EBB81-6DF6-4697-ADA4-2EE9B29406BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F86CFC26-5D52-4FBC-8579-18DF01C2A5C3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F86CFC26-5D52-4FBC-8579-18DF01C2A5C3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Procurement KPI Analysis Datase" sheetId="1" r:id="rId1"/>
+    <sheet name="Category Analysis" sheetId="3" r:id="rId1"/>
+    <sheet name="Supplier Analysis" sheetId="2" r:id="rId2"/>
+    <sheet name="Procurement KPI Analysis Datase" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Procurement KPI Analysis Datase'!$A$1:$Q$778</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Procurement KPI Analysis Datase'!$A$1:$Q$778</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3902" uniqueCount="810">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3936" uniqueCount="820">
   <si>
     <t>PO_ID</t>
   </si>
@@ -2466,6 +2468,36 @@
   </si>
   <si>
     <t>Delivery Days</t>
+  </si>
+  <si>
+    <t>Supplier Analysis</t>
+  </si>
+  <si>
+    <t>Supplier / Category</t>
+  </si>
+  <si>
+    <t>PO Count</t>
+  </si>
+  <si>
+    <t>Original Spend</t>
+  </si>
+  <si>
+    <t>Negotiated Spend</t>
+  </si>
+  <si>
+    <t>Defective Units</t>
+  </si>
+  <si>
+    <t>Compliant POs</t>
+  </si>
+  <si>
+    <t>Compliance Rate %</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Category Analysis</t>
   </si>
 </sst>
 </file>
@@ -3333,6 +3365,616 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4C4AC17-762D-44DB-9708-90FC0187A119}">
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>811</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>813</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>814</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>806</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>808</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$E:$E,"Electronics")</f>
+        <v>152</v>
+      </c>
+      <c r="C4">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Electronics",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>164829</v>
+      </c>
+      <c r="D4" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Electronics",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>9385426.8300000001</v>
+      </c>
+      <c r="E4" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Electronics",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>8642550.6000000071</v>
+      </c>
+      <c r="F4" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Electronics",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>742876.23</v>
+      </c>
+      <c r="G4">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Electronics",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>8981</v>
+      </c>
+      <c r="H4" s="3">
+        <f t="shared" ref="H4:H9" si="0">IFERROR(G4/C4,0)</f>
+        <v>5.4486771138573913E-2</v>
+      </c>
+      <c r="I4">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$E:$E,"Electronics",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>130</v>
+      </c>
+      <c r="J4" s="3">
+        <f t="shared" ref="J4:J9" si="1">IFERROR(I4/B4,0)</f>
+        <v>0.85526315789473684</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$E:$E,"MRO")</f>
+        <v>164</v>
+      </c>
+      <c r="C5">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"MRO",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>187658</v>
+      </c>
+      <c r="D5" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"MRO",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>11028921.170000004</v>
+      </c>
+      <c r="E5" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"MRO",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>10126608.859999996</v>
+      </c>
+      <c r="F5" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"MRO",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>902312.30999999982</v>
+      </c>
+      <c r="G5">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"MRO",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>9741</v>
+      </c>
+      <c r="H5" s="3">
+        <f t="shared" si="0"/>
+        <v>5.1908258640718755E-2</v>
+      </c>
+      <c r="I5">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$E:$E,"MRO",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>135</v>
+      </c>
+      <c r="J5" s="3">
+        <f t="shared" si="1"/>
+        <v>0.82317073170731703</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$E:$E,"Office Supplies")</f>
+        <v>174</v>
+      </c>
+      <c r="C6">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Office Supplies",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>179936</v>
+      </c>
+      <c r="D6" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Office Supplies",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>10851679.189999998</v>
+      </c>
+      <c r="E6" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Office Supplies",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>10007583.030000001</v>
+      </c>
+      <c r="F6" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Office Supplies",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>844096.16000000015</v>
+      </c>
+      <c r="G6">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Office Supplies",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>11233</v>
+      </c>
+      <c r="H6" s="3">
+        <f t="shared" si="0"/>
+        <v>6.2427752089631867E-2</v>
+      </c>
+      <c r="I6">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$E:$E,"Office Supplies",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>144</v>
+      </c>
+      <c r="J6" s="3">
+        <f t="shared" si="1"/>
+        <v>0.82758620689655171</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$E:$E,"Packaging")</f>
+        <v>148</v>
+      </c>
+      <c r="C7">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Packaging",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>166876</v>
+      </c>
+      <c r="D7" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Packaging",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>8858457.0000000056</v>
+      </c>
+      <c r="E7" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Packaging",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>8125712.4799999977</v>
+      </c>
+      <c r="F7" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Packaging",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>732744.52</v>
+      </c>
+      <c r="G7">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Packaging",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>8352</v>
+      </c>
+      <c r="H7" s="3">
+        <f t="shared" si="0"/>
+        <v>5.0049138282317412E-2</v>
+      </c>
+      <c r="I7">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$E:$E,"Packaging",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>118</v>
+      </c>
+      <c r="J7" s="3">
+        <f t="shared" si="1"/>
+        <v>0.79729729729729726</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$E:$E,"Raw Materials")</f>
+        <v>139</v>
+      </c>
+      <c r="C8">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Raw Materials",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>151252</v>
+      </c>
+      <c r="D8" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Raw Materials",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>9180338.6699999981</v>
+      </c>
+      <c r="E8" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Raw Materials",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>8471241.4199999999</v>
+      </c>
+      <c r="F8" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Raw Materials",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>709097.25000000035</v>
+      </c>
+      <c r="G8">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$E:$E,"Raw Materials",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>9642</v>
+      </c>
+      <c r="H8" s="3">
+        <f t="shared" si="0"/>
+        <v>6.3747917382910635E-2</v>
+      </c>
+      <c r="I8">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$E:$E,"Raw Materials",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>113</v>
+      </c>
+      <c r="J8" s="3">
+        <f t="shared" si="1"/>
+        <v>0.81294964028776984</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>818</v>
+      </c>
+      <c r="B9">
+        <f t="shared" ref="B9:G9" si="2">SUM(B4:B8)</f>
+        <v>777</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="2"/>
+        <v>850551</v>
+      </c>
+      <c r="D9" s="2">
+        <f t="shared" si="2"/>
+        <v>49304822.859999999</v>
+      </c>
+      <c r="E9" s="2">
+        <f t="shared" si="2"/>
+        <v>45373696.390000001</v>
+      </c>
+      <c r="F9" s="2">
+        <f t="shared" si="2"/>
+        <v>3931126.4700000007</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="2"/>
+        <v>47949</v>
+      </c>
+      <c r="H9" s="3">
+        <f t="shared" si="0"/>
+        <v>5.6374044589918772E-2</v>
+      </c>
+      <c r="I9">
+        <f>SUM(I4:I8)</f>
+        <v>640</v>
+      </c>
+      <c r="J9" s="3">
+        <f t="shared" si="1"/>
+        <v>0.82368082368082363</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33E2DD02-FF86-4238-84D3-87E7F43F7A78}">
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>811</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>813</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>814</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>806</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>808</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$B:$B,"Alpha_Inc")</f>
+        <v>141</v>
+      </c>
+      <c r="C4">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Alpha_Inc",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>150414</v>
+      </c>
+      <c r="D4" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Alpha_Inc",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>8528632.7400000002</v>
+      </c>
+      <c r="E4" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Alpha_Inc",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>7839712.2500000028</v>
+      </c>
+      <c r="F4" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Alpha_Inc",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>688920.49000000034</v>
+      </c>
+      <c r="G4">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Alpha_Inc",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>2717</v>
+      </c>
+      <c r="H4" s="3">
+        <f t="shared" ref="H4:H9" si="0">IFERROR(G4/C4,0)</f>
+        <v>1.8063478133684363E-2</v>
+      </c>
+      <c r="I4">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$B:$B,"Alpha_Inc",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>132</v>
+      </c>
+      <c r="J4" s="3">
+        <f t="shared" ref="J4:J9" si="1">IFERROR(I4/B4,0)</f>
+        <v>0.93617021276595747</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$B:$B,"Beta_Supplies")</f>
+        <v>156</v>
+      </c>
+      <c r="C5">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Beta_Supplies",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>180516</v>
+      </c>
+      <c r="D5" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Beta_Supplies",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>10748606.789999999</v>
+      </c>
+      <c r="E5" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Beta_Supplies",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>9858665.9000000022</v>
+      </c>
+      <c r="F5" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Beta_Supplies",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>889940.8900000006</v>
+      </c>
+      <c r="G5">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Beta_Supplies",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>13838</v>
+      </c>
+      <c r="H5" s="3">
+        <f t="shared" si="0"/>
+        <v>7.6658024773427286E-2</v>
+      </c>
+      <c r="I5">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$B:$B,"Beta_Supplies",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>118</v>
+      </c>
+      <c r="J5" s="3">
+        <f t="shared" si="1"/>
+        <v>0.75641025641025639</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$B:$B,"Delta_Logistics")</f>
+        <v>171</v>
+      </c>
+      <c r="C6">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Delta_Logistics",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>181652</v>
+      </c>
+      <c r="D6" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Delta_Logistics",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>10018216.960000006</v>
+      </c>
+      <c r="E6" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Delta_Logistics",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>9236240.4699999988</v>
+      </c>
+      <c r="F6" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Delta_Logistics",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>781976.49</v>
+      </c>
+      <c r="G6">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Delta_Logistics",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>19678</v>
+      </c>
+      <c r="H6" s="3">
+        <f t="shared" si="0"/>
+        <v>0.10832801180278775</v>
+      </c>
+      <c r="I6">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$B:$B,"Delta_Logistics",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>104</v>
+      </c>
+      <c r="J6" s="3">
+        <f t="shared" si="1"/>
+        <v>0.60818713450292394</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$B:$B,"Epsilon_Group")</f>
+        <v>166</v>
+      </c>
+      <c r="C7">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Epsilon_Group",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>180053</v>
+      </c>
+      <c r="D7" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Epsilon_Group",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>10696136.239999995</v>
+      </c>
+      <c r="E7" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Epsilon_Group",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>9851156.0600000024</v>
+      </c>
+      <c r="F7" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Epsilon_Group",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>844980.17999999982</v>
+      </c>
+      <c r="G7">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Epsilon_Group",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>4682</v>
+      </c>
+      <c r="H7" s="3">
+        <f t="shared" si="0"/>
+        <v>2.6003454538385921E-2</v>
+      </c>
+      <c r="I7">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$B:$B,"Epsilon_Group",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>163</v>
+      </c>
+      <c r="J7" s="3">
+        <f t="shared" si="1"/>
+        <v>0.98192771084337349</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <f>COUNTIF('Procurement KPI Analysis Datase'!$B:$B,"Gamma_Co")</f>
+        <v>143</v>
+      </c>
+      <c r="C8">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Gamma_Co",'Procurement KPI Analysis Datase'!$G:$G)</f>
+        <v>157916</v>
+      </c>
+      <c r="D8" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Gamma_Co",'Procurement KPI Analysis Datase'!$L:$L)</f>
+        <v>9313230.129999999</v>
+      </c>
+      <c r="E8" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Gamma_Co",'Procurement KPI Analysis Datase'!$M:$M)</f>
+        <v>8587921.7099999972</v>
+      </c>
+      <c r="F8" s="2">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Gamma_Co",'Procurement KPI Analysis Datase'!$N:$N)</f>
+        <v>725308.42000000027</v>
+      </c>
+      <c r="G8">
+        <f>SUMIF('Procurement KPI Analysis Datase'!$B:$B,"Gamma_Co",'Procurement KPI Analysis Datase'!$J:$J)</f>
+        <v>7034</v>
+      </c>
+      <c r="H8" s="3">
+        <f t="shared" si="0"/>
+        <v>4.4542668254008461E-2</v>
+      </c>
+      <c r="I8">
+        <f>COUNTIFS('Procurement KPI Analysis Datase'!$B:$B,"Gamma_Co",'Procurement KPI Analysis Datase'!$K:$K,"Yes")</f>
+        <v>123</v>
+      </c>
+      <c r="J8" s="3">
+        <f t="shared" si="1"/>
+        <v>0.8601398601398601</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>818</v>
+      </c>
+      <c r="B9">
+        <f t="shared" ref="B9:G9" si="2">SUM(B4:B8)</f>
+        <v>777</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="2"/>
+        <v>850551</v>
+      </c>
+      <c r="D9" s="2">
+        <f t="shared" si="2"/>
+        <v>49304822.859999999</v>
+      </c>
+      <c r="E9" s="2">
+        <f t="shared" si="2"/>
+        <v>45373696.390000001</v>
+      </c>
+      <c r="F9" s="2">
+        <f t="shared" si="2"/>
+        <v>3931126.4700000011</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="2"/>
+        <v>47949</v>
+      </c>
+      <c r="H9" s="3">
+        <f t="shared" si="0"/>
+        <v>5.6374044589918772E-2</v>
+      </c>
+      <c r="I9">
+        <f>SUM(I4:I8)</f>
+        <v>640</v>
+      </c>
+      <c r="J9" s="3">
+        <f t="shared" si="1"/>
+        <v>0.82368082368082363</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5768A551-3EE6-4F6B-B416-1F5F6091E6C0}">
   <dimension ref="A1:Q778"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Check formulas, dashboard, documentation, Git his-tory and presentation quality
</commit_message>
<xml_diff>
--- a/Excel/Procurement KPI Analysis Dataset.xlsx
+++ b/Excel/Procurement KPI Analysis Dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gebre\Desktop\Purchase-Order-Performance-Analysis\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77724DD1-3FA5-4066-B3AE-549BC1CE5B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49329414-1901-45E8-9C2C-024504DE4915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8880" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -2959,15 +2959,6 @@
     <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2990,10 +2981,8 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="15" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3006,6 +2995,17 @@
     <xf numFmtId="166" fontId="15" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3092,6 +3092,26 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="5"/>
+              <c:pt idx="0">
+                <c:v>Alpha_Inc</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Beta_Supplies</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Delta_Logistics</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Epsilon_Group</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>Gamma_Co</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Dashboard!$Q$31:$Q$35</c:f>
@@ -3117,39 +3137,6 @@
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-              <c15:filteredCategoryTitle>
-                <c15:cat>
-                  <c:strRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Dashboard!$P$31:$P$35</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:strCache>
-                      <c:ptCount val="5"/>
-                      <c:pt idx="0">
-                        <c:v>Alpha_Inc</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>Beta_Supplies</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>Delta_Logistics</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>Epsilon_Group</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>Gamma_Co</c:v>
-                      </c:pt>
-                    </c:strCache>
-                  </c:strRef>
-                </c15:cat>
-              </c15:filteredCategoryTitle>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-5FBD-4D93-B638-2B68EF232CE5}"/>
             </c:ext>
@@ -3178,6 +3165,26 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="5"/>
+              <c:pt idx="0">
+                <c:v>Alpha_Inc</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Beta_Supplies</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Delta_Logistics</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Epsilon_Group</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>Gamma_Co</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Dashboard!$R$31:$R$35</c:f>
@@ -3203,39 +3210,6 @@
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-              <c15:filteredCategoryTitle>
-                <c15:cat>
-                  <c:strRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Dashboard!$P$31:$P$35</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:strCache>
-                      <c:ptCount val="5"/>
-                      <c:pt idx="0">
-                        <c:v>Alpha_Inc</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>Beta_Supplies</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>Delta_Logistics</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>Epsilon_Group</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>Gamma_Co</c:v>
-                      </c:pt>
-                    </c:strCache>
-                  </c:strRef>
-                </c15:cat>
-              </c15:filteredCategoryTitle>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-5FBD-4D93-B638-2B68EF232CE5}"/>
             </c:ext>
@@ -3402,6 +3376,26 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="5"/>
+              <c:pt idx="0">
+                <c:v>Electronics</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>MRO</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Office Supplies</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Packaging</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>Raw Materials</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Dashboard!$U$31:$U$35</c:f>
@@ -3427,39 +3421,6 @@
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-              <c15:filteredCategoryTitle>
-                <c15:cat>
-                  <c:strRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Dashboard!$T$31:$T$35</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:strCache>
-                      <c:ptCount val="5"/>
-                      <c:pt idx="0">
-                        <c:v>Electronics</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>MRO</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>Office Supplies</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>Packaging</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>Raw Materials</c:v>
-                      </c:pt>
-                    </c:strCache>
-                  </c:strRef>
-                </c15:cat>
-              </c15:filteredCategoryTitle>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-4659-4A10-BCB1-C7A79A9947D8}"/>
             </c:ext>
@@ -3488,6 +3449,26 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="5"/>
+              <c:pt idx="0">
+                <c:v>Electronics</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>MRO</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Office Supplies</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Packaging</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>Raw Materials</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Dashboard!$V$31:$V$35</c:f>
@@ -3513,39 +3494,6 @@
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-              <c15:filteredCategoryTitle>
-                <c15:cat>
-                  <c:strRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Dashboard!$T$31:$T$35</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:strCache>
-                      <c:ptCount val="5"/>
-                      <c:pt idx="0">
-                        <c:v>Electronics</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>MRO</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>Office Supplies</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>Packaging</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>Raw Materials</c:v>
-                      </c:pt>
-                    </c:strCache>
-                  </c:strRef>
-                </c15:cat>
-              </c15:filteredCategoryTitle>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-4659-4A10-BCB1-C7A79A9947D8}"/>
             </c:ext>
@@ -3757,6 +3705,23 @@
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
             </c:extLst>
           </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="4"/>
+              <c:pt idx="0">
+                <c:v>Delivered</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Partially Delivered</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Pending</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Cancelled</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Dashboard!$Y$31:$Y$34</c:f>
@@ -3779,36 +3744,6 @@
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-              <c15:filteredCategoryTitle>
-                <c15:cat>
-                  <c:strRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Dashboard!$X$31:$X$34</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:strCache>
-                      <c:ptCount val="4"/>
-                      <c:pt idx="0">
-                        <c:v>Delivered</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>Partially Delivered</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>Pending</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>Cancelled</c:v>
-                      </c:pt>
-                    </c:strCache>
-                  </c:strRef>
-                </c15:cat>
-              </c15:filteredCategoryTitle>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-9334-480B-852D-C8A4F6D883F7}"/>
             </c:ext>
@@ -19871,59 +19806,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
     </row>
     <row r="2" spans="1:23" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
     </row>
     <row r="3" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="28"/>
-      <c r="M4" s="28"/>
-      <c r="N4" s="28"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
+      <c r="N4" s="35"/>
       <c r="S4" t="s">
         <v>887</v>
       </c>
@@ -19941,13 +19876,13 @@
       <c r="G5" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J5" s="27" t="s">
+      <c r="J5" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
+      <c r="K5" s="35"/>
+      <c r="L5" s="35"/>
+      <c r="M5" s="35"/>
+      <c r="N5" s="35"/>
     </row>
     <row r="6" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="24" t="s">
@@ -19962,11 +19897,11 @@
       <c r="H6" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="J6" s="28"/>
-      <c r="K6" s="28"/>
-      <c r="L6" s="28"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="35"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="35"/>
+      <c r="N6" s="35"/>
     </row>
     <row r="7" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="W7" t="s">
@@ -19975,85 +19910,85 @@
     </row>
     <row r="8" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="D9" s="38" t="s">
+      <c r="B9" s="30"/>
+      <c r="D9" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="G9" s="36" t="s">
+      <c r="E9" s="28"/>
+      <c r="G9" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="H9" s="37"/>
-      <c r="J9" s="36" t="s">
+      <c r="H9" s="32"/>
+      <c r="J9" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="K9" s="37"/>
-      <c r="M9" s="38" t="s">
+      <c r="K9" s="32"/>
+      <c r="M9" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="N9" s="33"/>
+      <c r="N9" s="28"/>
     </row>
     <row r="10" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="44">
+      <c r="A10" s="39">
         <f>SUMPRODUCT((('Procurement KPI Analysis Datase'!$B$2:$B$778=$B$6)+($B$6="All Suppliers"))*(('Procurement KPI Analysis Datase'!$E$2:$E$778=$D$6)+($D$6="All Categories"))*(('Procurement KPI Analysis Datase'!$F$2:$F$778=$F$6)+($F$6="All Statuses"))*(('Procurement KPI Analysis Datase'!$K$2:$K$778=$H$6)+($H$6="All Compliance"))*1)</f>
         <v>777</v>
       </c>
-      <c r="B10" s="35"/>
-      <c r="D10" s="32">
+      <c r="B10" s="30"/>
+      <c r="D10" s="27">
         <f>SUMPRODUCT((('Procurement KPI Analysis Datase'!$B$2:$B$778=$B$6)+($B$6="All Suppliers"))*(('Procurement KPI Analysis Datase'!$E$2:$E$778=$D$6)+($D$6="All Categories"))*(('Procurement KPI Analysis Datase'!$F$2:$F$778=$F$6)+($F$6="All Statuses"))*(('Procurement KPI Analysis Datase'!$K$2:$K$778=$H$6)+($H$6="All Compliance"))*('Procurement KPI Analysis Datase'!$M2:$M778))</f>
         <v>45373696.390000008</v>
       </c>
-      <c r="E10" s="33"/>
-      <c r="G10" s="42">
+      <c r="E10" s="28"/>
+      <c r="G10" s="37">
         <f>SUMPRODUCT((('Procurement KPI Analysis Datase'!$B$2:$B$778=$B$6)+($B$6="All Suppliers"))*(('Procurement KPI Analysis Datase'!$E$2:$E$778=$D$6)+($D$6="All Categories"))*(('Procurement KPI Analysis Datase'!$F$2:$F$778=$F$6)+($F$6="All Statuses"))*(('Procurement KPI Analysis Datase'!$K$2:$K$778=$H$6)+($H$6="All Compliance"))*('Procurement KPI Analysis Datase'!$N2:$N778))</f>
         <v>3931126.4699999993</v>
       </c>
-      <c r="H10" s="37"/>
-      <c r="J10" s="45">
+      <c r="H10" s="32"/>
+      <c r="J10" s="40">
         <f>IFERROR(G10/(G10+D10),0)</f>
         <v>7.9731073797026902E-2</v>
       </c>
-      <c r="K10" s="37"/>
-      <c r="M10" s="43">
+      <c r="K10" s="32"/>
+      <c r="M10" s="38">
         <f>IFERROR(SUMPRODUCT((('Procurement KPI Analysis Datase'!$B$2:$B$778=$B$6)+($B$6="All Suppliers"))*(('Procurement KPI Analysis Datase'!$E$2:$E$778=$D$6)+($D$6="All Categories"))*(('Procurement KPI Analysis Datase'!$F$2:$F$778=$F$6)+($F$6="All Statuses"))*(('Procurement KPI Analysis Datase'!$K$2:$K$778=$H$6)+($H$6="All Compliance"))*('Procurement KPI Analysis Datase'!$K$2:$K$778="Yes"))/A10,0)</f>
         <v>0.82368082368082363</v>
       </c>
-      <c r="N10" s="33"/>
+      <c r="N10" s="28"/>
     </row>
     <row r="11" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="35"/>
-      <c r="B11" s="35"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37"/>
-      <c r="J11" s="37"/>
-      <c r="K11" s="37"/>
-      <c r="M11" s="33"/>
-      <c r="N11" s="33"/>
+      <c r="A11" s="30"/>
+      <c r="B11" s="30"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+      <c r="M11" s="28"/>
+      <c r="N11" s="28"/>
     </row>
     <row r="12" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39" t="s">
+      <c r="A14" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
-      <c r="K14" s="28"/>
-      <c r="L14" s="28"/>
-      <c r="M14" s="28"/>
-      <c r="N14" s="28"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="35"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35"/>
+      <c r="J14" s="35"/>
+      <c r="K14" s="35"/>
+      <c r="L14" s="35"/>
+      <c r="M14" s="35"/>
+      <c r="N14" s="35"/>
     </row>
     <row r="15" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -20097,15 +20032,15 @@
       </c>
     </row>
     <row r="31" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H31" s="40" t="s">
+      <c r="H31" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="I31" s="28"/>
-      <c r="J31" s="28"/>
-      <c r="K31" s="28"/>
-      <c r="L31" s="28"/>
-      <c r="M31" s="28"/>
-      <c r="N31" s="28"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="35"/>
+      <c r="K31" s="35"/>
+      <c r="L31" s="35"/>
+      <c r="M31" s="35"/>
+      <c r="N31" s="35"/>
       <c r="P31" t="s">
         <v>18</v>
       </c>
@@ -20137,15 +20072,15 @@
       </c>
     </row>
     <row r="32" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H32" s="30" t="s">
+      <c r="H32" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="I32" s="31"/>
-      <c r="J32" s="31"/>
-      <c r="K32" s="31"/>
-      <c r="L32" s="31"/>
-      <c r="M32" s="31"/>
-      <c r="N32" s="31"/>
+      <c r="I32" s="26"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="26"/>
+      <c r="L32" s="26"/>
+      <c r="M32" s="26"/>
+      <c r="N32" s="26"/>
       <c r="P32" t="s">
         <v>21</v>
       </c>
@@ -20177,13 +20112,13 @@
       </c>
     </row>
     <row r="33" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H33" s="31"/>
-      <c r="I33" s="31"/>
-      <c r="J33" s="31"/>
-      <c r="K33" s="31"/>
-      <c r="L33" s="31"/>
-      <c r="M33" s="31"/>
-      <c r="N33" s="31"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="26"/>
+      <c r="J33" s="26"/>
+      <c r="K33" s="26"/>
+      <c r="L33" s="26"/>
+      <c r="M33" s="26"/>
+      <c r="N33" s="26"/>
       <c r="P33" t="s">
         <v>24</v>
       </c>
@@ -20215,13 +20150,13 @@
       </c>
     </row>
     <row r="34" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H34" s="31"/>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31"/>
-      <c r="K34" s="31"/>
-      <c r="L34" s="31"/>
-      <c r="M34" s="31"/>
-      <c r="N34" s="31"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="26"/>
+      <c r="J34" s="26"/>
+      <c r="K34" s="26"/>
+      <c r="L34" s="26"/>
+      <c r="M34" s="26"/>
+      <c r="N34" s="26"/>
       <c r="P34" t="s">
         <v>27</v>
       </c>
@@ -20253,13 +20188,13 @@
       </c>
     </row>
     <row r="35" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H35" s="31"/>
-      <c r="I35" s="31"/>
-      <c r="J35" s="31"/>
-      <c r="K35" s="31"/>
-      <c r="L35" s="31"/>
-      <c r="M35" s="31"/>
-      <c r="N35" s="31"/>
+      <c r="H35" s="26"/>
+      <c r="I35" s="26"/>
+      <c r="J35" s="26"/>
+      <c r="K35" s="26"/>
+      <c r="L35" s="26"/>
+      <c r="M35" s="26"/>
+      <c r="N35" s="26"/>
       <c r="P35" t="s">
         <v>30</v>
       </c>
@@ -20284,49 +20219,50 @@
       </c>
     </row>
     <row r="36" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H36" s="31"/>
-      <c r="I36" s="31"/>
-      <c r="J36" s="31"/>
-      <c r="K36" s="31"/>
-      <c r="L36" s="31"/>
-      <c r="M36" s="31"/>
-      <c r="N36" s="31"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="26"/>
+      <c r="J36" s="26"/>
+      <c r="K36" s="26"/>
+      <c r="L36" s="26"/>
+      <c r="M36" s="26"/>
+      <c r="N36" s="26"/>
     </row>
     <row r="37" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H37" s="31"/>
-      <c r="I37" s="31"/>
-      <c r="J37" s="31"/>
-      <c r="K37" s="31"/>
-      <c r="L37" s="31"/>
-      <c r="M37" s="31"/>
-      <c r="N37" s="31"/>
+      <c r="H37" s="26"/>
+      <c r="I37" s="26"/>
+      <c r="J37" s="26"/>
+      <c r="K37" s="26"/>
+      <c r="L37" s="26"/>
+      <c r="M37" s="26"/>
+      <c r="N37" s="26"/>
     </row>
     <row r="38" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H38" s="31"/>
-      <c r="I38" s="31"/>
-      <c r="J38" s="31"/>
-      <c r="K38" s="31"/>
-      <c r="L38" s="31"/>
-      <c r="M38" s="31"/>
-      <c r="N38" s="31"/>
+      <c r="H38" s="26"/>
+      <c r="I38" s="26"/>
+      <c r="J38" s="26"/>
+      <c r="K38" s="26"/>
+      <c r="L38" s="26"/>
+      <c r="M38" s="26"/>
+      <c r="N38" s="26"/>
     </row>
     <row r="39" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H39" s="31"/>
-      <c r="I39" s="31"/>
-      <c r="J39" s="31"/>
-      <c r="K39" s="31"/>
-      <c r="L39" s="31"/>
-      <c r="M39" s="31"/>
-      <c r="N39" s="31"/>
+      <c r="H39" s="26"/>
+      <c r="I39" s="26"/>
+      <c r="J39" s="26"/>
+      <c r="K39" s="26"/>
+      <c r="L39" s="26"/>
+      <c r="M39" s="26"/>
+      <c r="N39" s="26"/>
     </row>
     <row r="40" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="42" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="M9:N9"/>
     <mergeCell ref="J5:N6"/>
     <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A2:N2"/>
     <mergeCell ref="H32:N39"/>
     <mergeCell ref="D10:E11"/>
     <mergeCell ref="A9:B9"/>
@@ -20335,12 +20271,11 @@
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="A14:N14"/>
     <mergeCell ref="H31:N31"/>
-    <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A2:N2"/>
     <mergeCell ref="G10:H11"/>
     <mergeCell ref="M10:N11"/>
     <mergeCell ref="A10:B11"/>
     <mergeCell ref="J10:K11"/>
+    <mergeCell ref="M9:N9"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="list" errorTitle="Invalid filter" error="Choose a value from the list." sqref="B6" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -20999,25 +20934,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
@@ -21850,56 +21785,56 @@
       <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
       <c r="F4" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="28"/>
-      <c r="M4" s="28"/>
-      <c r="N4" s="28"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
+      <c r="N4" s="35"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">

</xml_diff>

<commit_message>
documentation and screen shoot image
</commit_message>
<xml_diff>
--- a/Excel/Procurement KPI Analysis Dataset.xlsx
+++ b/Excel/Procurement KPI Analysis Dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gebre\Desktop\Purchase-Order-Performance-Analysis\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49329414-1901-45E8-9C2C-024504DE4915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAD4357-8E35-48A1-B809-B5FDC131A14B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId7"/>
+    <pivotCache cacheId="2" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -2959,6 +2959,19 @@
     <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2978,10 +2991,6 @@
     <xf numFmtId="0" fontId="14" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="15" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2995,24 +3004,15 @@
     <xf numFmtId="166" fontId="15" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18741,7 +18741,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="ptQualityAnalysis" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="ptQualityAnalysis" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="A36:J44" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField dataField="1" showAll="0"/>
@@ -18924,11 +18924,11 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000004000000}" name="ptCostAnalysis" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000004000000}" name="ptCostAnalysis" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
   <location ref="J20:N27" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
       <items count="6">
         <item x="0"/>
         <item x="3"/>
@@ -18937,6 +18937,15 @@
         <item x="2"/>
         <item t="default"/>
       </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
     </pivotField>
     <pivotField numFmtId="14" showAll="0"/>
     <pivotField numFmtId="14" showAll="0"/>
@@ -18959,19 +18968,19 @@
   </rowFields>
   <rowItems count="6">
     <i>
-      <x/>
+      <x v="1"/>
     </i>
     <i>
-      <x v="1"/>
+      <x v="3"/>
     </i>
     <i>
       <x v="2"/>
     </i>
     <i>
-      <x v="3"/>
+      <x v="4"/>
     </i>
     <i>
-      <x v="4"/>
+      <x/>
     </i>
     <i t="grand">
       <x/>
@@ -19048,7 +19057,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000003000000}" name="ptStatusPerformance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000003000000}" name="ptStatusPerformance" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="A20:E26" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField dataField="1" showAll="0"/>
@@ -19056,7 +19065,7 @@
     <pivotField numFmtId="14" showAll="0"/>
     <pivotField numFmtId="14" showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
@@ -19064,6 +19073,15 @@
         <item x="3"/>
         <item t="default"/>
       </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -19082,16 +19100,16 @@
   </rowFields>
   <rowItems count="5">
     <i>
-      <x/>
+      <x v="1"/>
     </i>
     <i>
-      <x v="1"/>
+      <x v="3"/>
     </i>
     <i>
       <x v="2"/>
     </i>
     <i>
-      <x v="3"/>
+      <x/>
     </i>
     <i t="grand">
       <x/>
@@ -19168,7 +19186,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000002000000}" name="ptCategoryPerformance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000002000000}" name="ptCategoryPerformance" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
   <location ref="J4:P11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField dataField="1" showAll="0"/>
@@ -19318,7 +19336,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="ptSupplierPerformance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="ptSupplierPerformance" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="A4:G11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField dataField="1" showAll="0"/>
@@ -19806,59 +19824,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
     </row>
     <row r="2" spans="1:23" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
     </row>
     <row r="3" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="35"/>
-      <c r="K4" s="35"/>
-      <c r="L4" s="35"/>
-      <c r="M4" s="35"/>
-      <c r="N4" s="35"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
       <c r="S4" t="s">
         <v>887</v>
       </c>
@@ -19876,13 +19894,13 @@
       <c r="G5" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J5" s="41" t="s">
+      <c r="J5" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="K5" s="35"/>
-      <c r="L5" s="35"/>
-      <c r="M5" s="35"/>
-      <c r="N5" s="35"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="26"/>
     </row>
     <row r="6" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="24" t="s">
@@ -19897,11 +19915,11 @@
       <c r="H6" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="J6" s="35"/>
-      <c r="K6" s="35"/>
-      <c r="L6" s="35"/>
-      <c r="M6" s="35"/>
-      <c r="N6" s="35"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
     </row>
     <row r="7" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="W7" t="s">
@@ -19910,85 +19928,85 @@
     </row>
     <row r="8" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="30"/>
-      <c r="D9" s="33" t="s">
+      <c r="B9" s="35"/>
+      <c r="D9" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="28"/>
-      <c r="G9" s="31" t="s">
+      <c r="E9" s="33"/>
+      <c r="G9" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="H9" s="32"/>
-      <c r="J9" s="31" t="s">
+      <c r="H9" s="37"/>
+      <c r="J9" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="K9" s="32"/>
-      <c r="M9" s="33" t="s">
+      <c r="K9" s="37"/>
+      <c r="M9" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="N9" s="28"/>
+      <c r="N9" s="33"/>
     </row>
     <row r="10" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="39">
+      <c r="A10" s="42">
         <f>SUMPRODUCT((('Procurement KPI Analysis Datase'!$B$2:$B$778=$B$6)+($B$6="All Suppliers"))*(('Procurement KPI Analysis Datase'!$E$2:$E$778=$D$6)+($D$6="All Categories"))*(('Procurement KPI Analysis Datase'!$F$2:$F$778=$F$6)+($F$6="All Statuses"))*(('Procurement KPI Analysis Datase'!$K$2:$K$778=$H$6)+($H$6="All Compliance"))*1)</f>
         <v>777</v>
       </c>
-      <c r="B10" s="30"/>
-      <c r="D10" s="27">
+      <c r="B10" s="35"/>
+      <c r="D10" s="32">
         <f>SUMPRODUCT((('Procurement KPI Analysis Datase'!$B$2:$B$778=$B$6)+($B$6="All Suppliers"))*(('Procurement KPI Analysis Datase'!$E$2:$E$778=$D$6)+($D$6="All Categories"))*(('Procurement KPI Analysis Datase'!$F$2:$F$778=$F$6)+($F$6="All Statuses"))*(('Procurement KPI Analysis Datase'!$K$2:$K$778=$H$6)+($H$6="All Compliance"))*('Procurement KPI Analysis Datase'!$M2:$M778))</f>
         <v>45373696.390000008</v>
       </c>
-      <c r="E10" s="28"/>
-      <c r="G10" s="37">
+      <c r="E10" s="33"/>
+      <c r="G10" s="40">
         <f>SUMPRODUCT((('Procurement KPI Analysis Datase'!$B$2:$B$778=$B$6)+($B$6="All Suppliers"))*(('Procurement KPI Analysis Datase'!$E$2:$E$778=$D$6)+($D$6="All Categories"))*(('Procurement KPI Analysis Datase'!$F$2:$F$778=$F$6)+($F$6="All Statuses"))*(('Procurement KPI Analysis Datase'!$K$2:$K$778=$H$6)+($H$6="All Compliance"))*('Procurement KPI Analysis Datase'!$N2:$N778))</f>
         <v>3931126.4699999993</v>
       </c>
-      <c r="H10" s="32"/>
-      <c r="J10" s="40">
+      <c r="H10" s="37"/>
+      <c r="J10" s="43">
         <f>IFERROR(G10/(G10+D10),0)</f>
         <v>7.9731073797026902E-2</v>
       </c>
-      <c r="K10" s="32"/>
-      <c r="M10" s="38">
+      <c r="K10" s="37"/>
+      <c r="M10" s="41">
         <f>IFERROR(SUMPRODUCT((('Procurement KPI Analysis Datase'!$B$2:$B$778=$B$6)+($B$6="All Suppliers"))*(('Procurement KPI Analysis Datase'!$E$2:$E$778=$D$6)+($D$6="All Categories"))*(('Procurement KPI Analysis Datase'!$F$2:$F$778=$F$6)+($F$6="All Statuses"))*(('Procurement KPI Analysis Datase'!$K$2:$K$778=$H$6)+($H$6="All Compliance"))*('Procurement KPI Analysis Datase'!$K$2:$K$778="Yes"))/A10,0)</f>
         <v>0.82368082368082363</v>
       </c>
-      <c r="N10" s="28"/>
+      <c r="N10" s="33"/>
     </row>
     <row r="11" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="30"/>
-      <c r="B11" s="30"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="J11" s="32"/>
-      <c r="K11" s="32"/>
-      <c r="M11" s="28"/>
-      <c r="N11" s="28"/>
+      <c r="A11" s="35"/>
+      <c r="B11" s="35"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="37"/>
+      <c r="J11" s="37"/>
+      <c r="K11" s="37"/>
+      <c r="M11" s="33"/>
+      <c r="N11" s="33"/>
     </row>
     <row r="12" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="34" t="s">
+      <c r="A14" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="35"/>
-      <c r="L14" s="35"/>
-      <c r="M14" s="35"/>
-      <c r="N14" s="35"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="26"/>
+      <c r="K14" s="26"/>
+      <c r="L14" s="26"/>
+      <c r="M14" s="26"/>
+      <c r="N14" s="26"/>
     </row>
     <row r="15" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -20032,15 +20050,15 @@
       </c>
     </row>
     <row r="31" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H31" s="36" t="s">
+      <c r="H31" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="I31" s="35"/>
-      <c r="J31" s="35"/>
-      <c r="K31" s="35"/>
-      <c r="L31" s="35"/>
-      <c r="M31" s="35"/>
-      <c r="N31" s="35"/>
+      <c r="I31" s="26"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="26"/>
+      <c r="L31" s="26"/>
+      <c r="M31" s="26"/>
+      <c r="N31" s="26"/>
       <c r="P31" t="s">
         <v>18</v>
       </c>
@@ -20072,15 +20090,15 @@
       </c>
     </row>
     <row r="32" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H32" s="25" t="s">
+      <c r="H32" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="26"/>
+      <c r="I32" s="31"/>
+      <c r="J32" s="31"/>
+      <c r="K32" s="31"/>
+      <c r="L32" s="31"/>
+      <c r="M32" s="31"/>
+      <c r="N32" s="31"/>
       <c r="P32" t="s">
         <v>21</v>
       </c>
@@ -20112,13 +20130,13 @@
       </c>
     </row>
     <row r="33" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
-      <c r="K33" s="26"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="26"/>
-      <c r="N33" s="26"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="31"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31"/>
+      <c r="L33" s="31"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="31"/>
       <c r="P33" t="s">
         <v>24</v>
       </c>
@@ -20150,13 +20168,13 @@
       </c>
     </row>
     <row r="34" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="26"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="26"/>
-      <c r="M34" s="26"/>
-      <c r="N34" s="26"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="31"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="31"/>
+      <c r="M34" s="31"/>
+      <c r="N34" s="31"/>
       <c r="P34" t="s">
         <v>27</v>
       </c>
@@ -20188,13 +20206,13 @@
       </c>
     </row>
     <row r="35" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H35" s="26"/>
-      <c r="I35" s="26"/>
-      <c r="J35" s="26"/>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="26"/>
-      <c r="N35" s="26"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="31"/>
+      <c r="L35" s="31"/>
+      <c r="M35" s="31"/>
+      <c r="N35" s="31"/>
       <c r="P35" t="s">
         <v>30</v>
       </c>
@@ -20219,46 +20237,47 @@
       </c>
     </row>
     <row r="36" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H36" s="26"/>
-      <c r="I36" s="26"/>
-      <c r="J36" s="26"/>
-      <c r="K36" s="26"/>
-      <c r="L36" s="26"/>
-      <c r="M36" s="26"/>
-      <c r="N36" s="26"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="31"/>
+      <c r="J36" s="31"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="31"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="31"/>
     </row>
     <row r="37" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
-      <c r="K37" s="26"/>
-      <c r="L37" s="26"/>
-      <c r="M37" s="26"/>
-      <c r="N37" s="26"/>
+      <c r="H37" s="31"/>
+      <c r="I37" s="31"/>
+      <c r="J37" s="31"/>
+      <c r="K37" s="31"/>
+      <c r="L37" s="31"/>
+      <c r="M37" s="31"/>
+      <c r="N37" s="31"/>
     </row>
     <row r="38" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
-      <c r="J38" s="26"/>
-      <c r="K38" s="26"/>
-      <c r="L38" s="26"/>
-      <c r="M38" s="26"/>
-      <c r="N38" s="26"/>
+      <c r="H38" s="31"/>
+      <c r="I38" s="31"/>
+      <c r="J38" s="31"/>
+      <c r="K38" s="31"/>
+      <c r="L38" s="31"/>
+      <c r="M38" s="31"/>
+      <c r="N38" s="31"/>
     </row>
     <row r="39" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H39" s="26"/>
-      <c r="I39" s="26"/>
-      <c r="J39" s="26"/>
-      <c r="K39" s="26"/>
-      <c r="L39" s="26"/>
-      <c r="M39" s="26"/>
-      <c r="N39" s="26"/>
+      <c r="H39" s="31"/>
+      <c r="I39" s="31"/>
+      <c r="J39" s="31"/>
+      <c r="K39" s="31"/>
+      <c r="L39" s="31"/>
+      <c r="M39" s="31"/>
+      <c r="N39" s="31"/>
     </row>
     <row r="40" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="42" spans="8:25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="M9:N9"/>
     <mergeCell ref="J5:N6"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A4:N4"/>
@@ -20275,7 +20294,6 @@
     <mergeCell ref="M10:N11"/>
     <mergeCell ref="A10:B11"/>
     <mergeCell ref="J10:K11"/>
-    <mergeCell ref="M9:N9"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="list" errorTitle="Invalid filter" error="Choose a value from the list." sqref="B6" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -20912,16 +20930,16 @@
   <dimension ref="A1:Q53"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.21875" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.5546875" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.21875" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.21875" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="24.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.77734375" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" style="6" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
@@ -21284,12 +21302,20 @@
     <row r="18" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="19" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="20" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20"/>
       <c r="B20" s="8" t="s">
         <v>87</v>
       </c>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="J20"/>
       <c r="K20" s="8" t="s">
         <v>87</v>
       </c>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
     </row>
     <row r="21" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -21325,66 +21351,66 @@
     </row>
     <row r="22" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B22" s="10">
-        <v>63</v>
+        <v>560</v>
       </c>
       <c r="C22" s="2">
-        <v>3882701.5100000012</v>
+        <v>35169009.019999966</v>
       </c>
       <c r="D22" s="2">
-        <v>3590495.1199999992</v>
+        <v>32408662.819999989</v>
       </c>
       <c r="E22" s="11">
-        <v>11.74603174603175</v>
+        <v>10.553571428571429</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="K22" s="2">
-        <v>8528632.7400000002</v>
+        <v>10748606.789999999</v>
       </c>
       <c r="L22" s="2">
-        <v>7839712.2500000028</v>
+        <v>9858665.9000000022</v>
       </c>
       <c r="M22" s="2">
-        <v>688920.49000000034</v>
+        <v>889940.89000000036</v>
       </c>
       <c r="N22" s="3">
-        <v>8.2104590467255753E-2</v>
+        <v>7.8276992247910529E-2</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B23" s="10">
-        <v>560</v>
+        <v>81</v>
       </c>
       <c r="C23" s="2">
-        <v>35169009.019999973</v>
+        <v>5852067.3999999994</v>
       </c>
       <c r="D23" s="2">
-        <v>32408662.819999989</v>
+        <v>5306302.3099999987</v>
       </c>
       <c r="E23" s="11">
-        <v>10.553571428571431</v>
+        <v>11.938271604938272</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K23" s="2">
-        <v>10748606.789999999</v>
+        <v>10696136.239999995</v>
       </c>
       <c r="L23" s="2">
-        <v>9858665.9000000022</v>
+        <v>9851156.0600000042</v>
       </c>
       <c r="M23" s="2">
-        <v>889940.8900000006</v>
+        <v>844980.1799999997</v>
       </c>
       <c r="N23" s="3">
-        <v>7.8276992247910543E-2</v>
+        <v>8.0405205072453911E-2</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -21398,22 +21424,22 @@
         <v>4401044.9300000006</v>
       </c>
       <c r="D24" s="2">
-        <v>4068236.14</v>
+        <v>4068236.1399999997</v>
       </c>
       <c r="E24" s="11">
-        <v>11.013698630136989</v>
+        <v>11.013698630136986</v>
       </c>
       <c r="J24" s="9" t="s">
         <v>24</v>
       </c>
       <c r="K24" s="2">
-        <v>10018216.96000001</v>
+        <v>10018216.960000006</v>
       </c>
       <c r="L24" s="2">
         <v>9236240.4699999988</v>
       </c>
       <c r="M24" s="2">
-        <v>781976.49</v>
+        <v>781976.48999999987</v>
       </c>
       <c r="N24" s="3">
         <v>7.811976922617335E-2</v>
@@ -21421,34 +21447,34 @@
     </row>
     <row r="25" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="10">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C25" s="2">
-        <v>5852067.3999999994</v>
+        <v>3882701.5100000007</v>
       </c>
       <c r="D25" s="2">
-        <v>5306302.3099999987</v>
+        <v>3590495.1199999992</v>
       </c>
       <c r="E25" s="11">
-        <v>11.93827160493827</v>
+        <v>11.746031746031745</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="K25" s="2">
-        <v>10696136.239999991</v>
+        <v>9313230.129999999</v>
       </c>
       <c r="L25" s="2">
-        <v>9851156.0600000024</v>
+        <v>8587921.7099999972</v>
       </c>
       <c r="M25" s="2">
-        <v>844980.17999999982</v>
+        <v>725308.42000000027</v>
       </c>
       <c r="N25" s="3">
-        <v>8.0405205072453925E-2</v>
+        <v>7.9848562374747037E-2</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -21462,25 +21488,25 @@
         <v>49304822.859999962</v>
       </c>
       <c r="D26" s="2">
-        <v>45373696.389999993</v>
+        <v>45373696.389999986</v>
       </c>
       <c r="E26" s="11">
-        <v>10.83783783783784</v>
+        <v>10.837837837837839</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="K26" s="2">
-        <v>9313230.129999999</v>
+        <v>8528632.7400000002</v>
       </c>
       <c r="L26" s="2">
-        <v>8587921.7099999972</v>
+        <v>7839712.2500000028</v>
       </c>
       <c r="M26" s="2">
-        <v>725308.42000000027</v>
+        <v>688920.49000000022</v>
       </c>
       <c r="N26" s="3">
-        <v>7.9848562374747037E-2</v>
+        <v>8.2104590467255753E-2</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -21488,13 +21514,13 @@
         <v>91</v>
       </c>
       <c r="K27" s="2">
-        <v>49304822.859999977</v>
+        <v>49304822.859999985</v>
       </c>
       <c r="L27" s="2">
-        <v>45373696.390000023</v>
+        <v>45373696.390000015</v>
       </c>
       <c r="M27" s="2">
-        <v>3931126.469999996</v>
+        <v>3931126.4699999951</v>
       </c>
       <c r="N27" s="3">
         <v>7.9680884228891843E-2</v>
@@ -21782,59 +21808,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="23.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="F4" s="48" t="s">
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="F4" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="35"/>
-      <c r="K4" s="35"/>
-      <c r="L4" s="35"/>
-      <c r="M4" s="35"/>
-      <c r="N4" s="35"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
@@ -21843,10 +21869,10 @@
       <c r="B5" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="49" t="s">
+      <c r="C5" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="47"/>
+      <c r="D5" s="46"/>
       <c r="E5" s="13"/>
       <c r="F5" s="12" t="s">
         <v>7</v>
@@ -21884,10 +21910,10 @@
         <f>COUNTA('Procurement KPI Analysis Datase'!$A$2:$A$778)</f>
         <v>777</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="47"/>
+      <c r="D6" s="46"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14" t="s">
         <v>18</v>
@@ -21933,10 +21959,10 @@
         <f>SUM('Procurement KPI Analysis Datase'!$G$2:$G$778)</f>
         <v>850551</v>
       </c>
-      <c r="C7" s="47" t="s">
+      <c r="C7" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="47"/>
+      <c r="D7" s="46"/>
       <c r="E7" s="13"/>
       <c r="F7" s="13" t="s">
         <v>21</v>
@@ -21982,10 +22008,10 @@
         <f>SUM('Procurement KPI Analysis Datase'!$L$2:$L$778)</f>
         <v>49304822.85999997</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="47"/>
+      <c r="D8" s="46"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14" t="s">
         <v>24</v>
@@ -22031,10 +22057,10 @@
         <f>SUM('Procurement KPI Analysis Datase'!$M$2:$M$778)</f>
         <v>45373696.390000008</v>
       </c>
-      <c r="C9" s="47" t="s">
+      <c r="C9" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="47"/>
+      <c r="D9" s="46"/>
       <c r="E9" s="13"/>
       <c r="F9" s="13" t="s">
         <v>27</v>
@@ -22080,10 +22106,10 @@
         <f>SUM('Procurement KPI Analysis Datase'!$N$2:$N$778)</f>
         <v>3931126.4699999993</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="48" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="47"/>
+      <c r="D10" s="46"/>
       <c r="E10" s="14"/>
       <c r="F10" s="14" t="s">
         <v>30</v>
@@ -22129,10 +22155,10 @@
         <f>IFERROR(B10/B8,0)</f>
         <v>7.9731073797026958E-2</v>
       </c>
-      <c r="C11" s="47" t="s">
+      <c r="C11" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="47"/>
+      <c r="D11" s="46"/>
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
@@ -22152,10 +22178,10 @@
         <f>AVERAGE('Procurement KPI Analysis Datase'!$O$2:$O$778)</f>
         <v>7.9680884228891816E-2</v>
       </c>
-      <c r="C12" s="46" t="s">
+      <c r="C12" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="47"/>
+      <c r="D12" s="46"/>
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
       <c r="G12" s="14"/>
@@ -22175,22 +22201,22 @@
         <f>AVERAGE('Procurement KPI Analysis Datase'!$Q$2:$Q$778)</f>
         <v>10.837837837837839</v>
       </c>
-      <c r="C13" s="47" t="s">
+      <c r="C13" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="47"/>
+      <c r="D13" s="46"/>
       <c r="E13" s="13"/>
-      <c r="F13" s="51" t="s">
+      <c r="F13" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="G13" s="47"/>
-      <c r="H13" s="47"/>
-      <c r="I13" s="47"/>
-      <c r="J13" s="47"/>
-      <c r="K13" s="47"/>
-      <c r="L13" s="47"/>
-      <c r="M13" s="47"/>
-      <c r="N13" s="47"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="46"/>
+      <c r="I13" s="46"/>
+      <c r="J13" s="46"/>
+      <c r="K13" s="46"/>
+      <c r="L13" s="46"/>
+      <c r="M13" s="46"/>
+      <c r="N13" s="46"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
@@ -22200,19 +22226,19 @@
         <f>SUM('Procurement KPI Analysis Datase'!$J$2:$J$778)/SUM('Procurement KPI Analysis Datase'!$G$2:$G$778)</f>
         <v>5.6374044589918772E-2</v>
       </c>
-      <c r="C14" s="46" t="s">
+      <c r="C14" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="47"/>
+      <c r="D14" s="46"/>
       <c r="E14" s="14"/>
       <c r="F14" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="G14" s="46" t="s">
+      <c r="G14" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="H14" s="47"/>
-      <c r="I14" s="47"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
       <c r="J14" s="14"/>
       <c r="K14" s="14"/>
       <c r="L14" s="14"/>
@@ -22227,19 +22253,19 @@
         <f>COUNTIF('Procurement KPI Analysis Datase'!$K$2:$K$778,"Yes")/COUNTA('Procurement KPI Analysis Datase'!$A$2:$A$778)</f>
         <v>0.82368082368082363</v>
       </c>
-      <c r="C15" s="47" t="s">
+      <c r="C15" s="46" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="47"/>
+      <c r="D15" s="46"/>
       <c r="E15" s="13"/>
       <c r="F15" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="47" t="s">
+      <c r="G15" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="H15" s="47"/>
-      <c r="I15" s="47"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
       <c r="J15" s="13"/>
       <c r="K15" s="13"/>
       <c r="L15" s="13"/>
@@ -22254,19 +22280,19 @@
         <f>COUNTIF('Procurement KPI Analysis Datase'!$F$2:$F$778,"Delivered")/COUNTA('Procurement KPI Analysis Datase'!$A$2:$A$778)</f>
         <v>0.72072072072072069</v>
       </c>
-      <c r="C16" s="46" t="s">
+      <c r="C16" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="47"/>
+      <c r="D16" s="46"/>
       <c r="E16" s="14"/>
       <c r="F16" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="G16" s="46" t="s">
+      <c r="G16" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="47"/>
-      <c r="I16" s="47"/>
+      <c r="H16" s="46"/>
+      <c r="I16" s="46"/>
       <c r="J16" s="14"/>
       <c r="K16" s="14"/>
       <c r="L16" s="14"/>
@@ -22282,11 +22308,11 @@
       <c r="F17" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="G17" s="47" t="s">
+      <c r="G17" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="H17" s="47"/>
-      <c r="I17" s="47"/>
+      <c r="H17" s="46"/>
+      <c r="I17" s="46"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13"/>
       <c r="L17" s="13"/>
@@ -22295,6 +22321,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C14:D14"/>
     <mergeCell ref="G17:I17"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="G15:I15"/>
@@ -22311,11 +22342,6 @@
     <mergeCell ref="F4:N4"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>